<commit_message>
Manage BOM template lines and remove filters
</commit_message>
<xml_diff>
--- a/Template_BOQ.xlsx
+++ b/Template_BOQ.xlsx
@@ -59,739 +59,739 @@
     <t>Menu colonna G</t>
   </si>
   <si>
+    <t>ARUHP</t>
+  </si>
+  <si>
+    <t>30 CURVA</t>
+  </si>
+  <si>
+    <t>*</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>GTS</t>
+  </si>
+  <si>
+    <t>CDA</t>
+  </si>
+  <si>
+    <t>45 CURVA</t>
+  </si>
+  <si>
+    <t>ARMANO</t>
+  </si>
+  <si>
+    <t>10</t>
+  </si>
+  <si>
+    <t>Linde</t>
+  </si>
+  <si>
+    <t>CDA-01</t>
+  </si>
+  <si>
+    <t>90 CURVA</t>
+  </si>
+  <si>
+    <t>COAX</t>
+  </si>
+  <si>
+    <t>100</t>
+  </si>
+  <si>
+    <t>CDA-02</t>
+  </si>
+  <si>
+    <t>BOCCHETTONE</t>
+  </si>
+  <si>
+    <t>CRISTAL</t>
+  </si>
+  <si>
+    <t>100X44,5</t>
+  </si>
+  <si>
+    <t>CF4</t>
+  </si>
+  <si>
+    <t>BOCCHETTONI</t>
+  </si>
+  <si>
+    <t>CUSTOM</t>
+  </si>
+  <si>
+    <t>100X80</t>
+  </si>
+  <si>
+    <t>CH2F2</t>
+  </si>
+  <si>
+    <t>BULK HEAD</t>
+  </si>
+  <si>
+    <t>DKW</t>
+  </si>
+  <si>
+    <t>104</t>
+  </si>
+  <si>
+    <t>CH3F</t>
+  </si>
+  <si>
+    <t>BUSSOLA DI RIDUZIONE</t>
+  </si>
+  <si>
+    <t>EP</t>
+  </si>
+  <si>
+    <t>10MMX1/2</t>
+  </si>
+  <si>
+    <t>CH4</t>
+  </si>
+  <si>
+    <t>CALOTTA</t>
+  </si>
+  <si>
+    <t>EVANS</t>
+  </si>
+  <si>
+    <t>110</t>
+  </si>
+  <si>
+    <t>CHF3</t>
+  </si>
+  <si>
+    <t>CANALINA CABLOFIL</t>
+  </si>
+  <si>
+    <t>GEMU</t>
+  </si>
+  <si>
+    <t>110X90</t>
+  </si>
+  <si>
+    <t>CL2</t>
+  </si>
+  <si>
+    <t>CARTELLA + FLANGIA (ACC+PPH)</t>
+  </si>
+  <si>
+    <t>HAMLET</t>
+  </si>
+  <si>
+    <t>1,1/2</t>
+  </si>
+  <si>
+    <t>CO2</t>
+  </si>
+  <si>
+    <t>CIECA</t>
+  </si>
+  <si>
+    <t>INOX</t>
+  </si>
+  <si>
+    <t>1,1/2X1</t>
+  </si>
+  <si>
+    <t>CT LIM</t>
+  </si>
+  <si>
+    <t>CURVA</t>
+  </si>
+  <si>
+    <t>JACOB</t>
+  </si>
+  <si>
+    <t>1,1/2X1/2</t>
+  </si>
+  <si>
+    <t>CT WATER</t>
+  </si>
+  <si>
+    <t>CURVE</t>
+  </si>
+  <si>
+    <t>PARKER</t>
+  </si>
+  <si>
+    <t>1,1/2X1/4</t>
+  </si>
+  <si>
+    <t>DRDA-01</t>
+  </si>
+  <si>
+    <t>DADO + FERULE ANT E POST</t>
+  </si>
+  <si>
+    <t>PFA</t>
+  </si>
+  <si>
+    <t>1,1/2X3/4</t>
+  </si>
+  <si>
+    <t>DRDA-02</t>
+  </si>
+  <si>
+    <t>FEMALE GLAND</t>
+  </si>
+  <si>
+    <t>PPH</t>
+  </si>
+  <si>
+    <t>1,1/2X38</t>
+  </si>
+  <si>
+    <t>DRDHF</t>
+  </si>
+  <si>
+    <t>FEMAL GLAND</t>
+  </si>
+  <si>
+    <t>PTFE</t>
+  </si>
+  <si>
+    <t>1,1/2X3/8</t>
+  </si>
+  <si>
+    <t>DRHF-01</t>
+  </si>
+  <si>
+    <t>FLANGIA</t>
+  </si>
+  <si>
+    <t>PVC</t>
+  </si>
+  <si>
+    <t>1,1/2X38,1</t>
+  </si>
+  <si>
+    <t>DRHF-02</t>
+  </si>
+  <si>
+    <t>FLANGIA CIECA</t>
+  </si>
+  <si>
+    <t>PVDF</t>
+  </si>
+  <si>
+    <t>1,1/4</t>
+  </si>
+  <si>
+    <t>DRNH-01</t>
+  </si>
+  <si>
+    <t>FLANGIA CLAMP</t>
+  </si>
+  <si>
+    <t>PVDF STD</t>
+  </si>
+  <si>
+    <t>1/2</t>
+  </si>
+  <si>
+    <t>DRNH-02</t>
+  </si>
+  <si>
+    <t>FLANGIA CUSTOM</t>
+  </si>
+  <si>
+    <t>PVDF UHP</t>
+  </si>
+  <si>
+    <t>1/2X10MM (M)</t>
+  </si>
+  <si>
+    <t>DRREC-01</t>
+  </si>
+  <si>
+    <t>FLANGIA DI PARTENZA DA POC</t>
+  </si>
+  <si>
+    <t>PVDF VENT</t>
+  </si>
+  <si>
+    <t>1/2X1/4</t>
+  </si>
+  <si>
+    <t>DRSOLF</t>
+  </si>
+  <si>
+    <t>FLANGIA KF</t>
+  </si>
+  <si>
+    <t>RILSAN</t>
+  </si>
+  <si>
+    <t>1/2X3/8</t>
+  </si>
+  <si>
+    <t>EXAC</t>
+  </si>
+  <si>
+    <t>FLANGIA KF CUSTOM</t>
+  </si>
+  <si>
+    <t>SMC</t>
+  </si>
+  <si>
+    <t>1/4</t>
+  </si>
+  <si>
+    <t>EXAC-01</t>
+  </si>
+  <si>
+    <t>FLANGIA PP/ACC + CARTELLA + GUARN PTFE</t>
+  </si>
+  <si>
+    <t>SPECTRON</t>
+  </si>
+  <si>
+    <t>140</t>
+  </si>
+  <si>
+    <t>EXHE 01</t>
+  </si>
+  <si>
+    <t>FLANGIA TPOC</t>
+  </si>
+  <si>
+    <t>STREAS</t>
+  </si>
+  <si>
+    <t>1/4MX1/2</t>
+  </si>
+  <si>
+    <t>EXHE 02</t>
+  </si>
+  <si>
+    <t>FLK</t>
+  </si>
+  <si>
+    <t>TASSALINI</t>
+  </si>
+  <si>
+    <t>1/4X1/2</t>
+  </si>
+  <si>
+    <t>EXNH-01</t>
+  </si>
+  <si>
+    <t>FLK FEMMINA ( GHIERA GIREVOLE )</t>
+  </si>
+  <si>
+    <t>TCC</t>
+  </si>
+  <si>
+    <t>150</t>
+  </si>
+  <si>
+    <t>EXNH02</t>
+  </si>
+  <si>
+    <t>FLOW METER</t>
+  </si>
+  <si>
+    <t>VCR</t>
+  </si>
+  <si>
+    <t>160</t>
+  </si>
+  <si>
+    <t>H2</t>
+  </si>
+  <si>
+    <t>FLOW METER CLAMPATO</t>
+  </si>
+  <si>
+    <t>ZINCATA</t>
+  </si>
+  <si>
+    <t>1"X1/2</t>
+  </si>
+  <si>
+    <t>HBr</t>
+  </si>
+  <si>
+    <t>FLUSSIMETRO CLAMPATO</t>
+  </si>
+  <si>
+    <t>1X32</t>
+  </si>
+  <si>
+    <t>HeUHP</t>
+  </si>
+  <si>
+    <t>FONDELLO</t>
+  </si>
+  <si>
+    <t>1X3/4</t>
+  </si>
+  <si>
+    <t>LIM 01,,12</t>
+  </si>
+  <si>
+    <t>GASKET INOX</t>
+  </si>
+  <si>
+    <t>1X3/8</t>
+  </si>
+  <si>
+    <t>LIM 1…20</t>
+  </si>
+  <si>
+    <t>GASKET NICHEL</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
     <t>linea</t>
   </si>
   <si>
-    <t>30 CURVA</t>
-  </si>
-  <si>
-    <t>*</t>
-  </si>
-  <si>
-    <t>1</t>
-  </si>
-  <si>
-    <t>GTS</t>
-  </si>
-  <si>
-    <t>ARUHP</t>
-  </si>
-  <si>
-    <t>45 CURVA</t>
-  </si>
-  <si>
-    <t>ARMANO</t>
-  </si>
-  <si>
-    <t>10</t>
-  </si>
-  <si>
-    <t>Linde</t>
-  </si>
-  <si>
-    <t>CO2</t>
-  </si>
-  <si>
-    <t>90 CURVA</t>
-  </si>
-  <si>
-    <t>COAX</t>
-  </si>
-  <si>
-    <t>100</t>
-  </si>
-  <si>
-    <t>CDA</t>
-  </si>
-  <si>
-    <t>BOCCHETTONE</t>
-  </si>
-  <si>
-    <t>CRISTAL</t>
-  </si>
-  <si>
-    <t>100X44,5</t>
-  </si>
-  <si>
-    <t>CF4</t>
-  </si>
-  <si>
-    <t>BOCCHETTONI</t>
-  </si>
-  <si>
-    <t>CUSTOM</t>
-  </si>
-  <si>
-    <t>100X80</t>
-  </si>
-  <si>
-    <t>CH2F2</t>
-  </si>
-  <si>
-    <t>BULK HEAD</t>
-  </si>
-  <si>
-    <t>DKW</t>
-  </si>
-  <si>
-    <t>104</t>
-  </si>
-  <si>
-    <t>CH3F</t>
-  </si>
-  <si>
-    <t>BUSSOLA DI RIDUZIONE</t>
-  </si>
-  <si>
-    <t>EP</t>
-  </si>
-  <si>
-    <t>10MMX1/2</t>
-  </si>
-  <si>
-    <t>CH4</t>
-  </si>
-  <si>
-    <t>CALOTTA</t>
-  </si>
-  <si>
-    <t>EVANS</t>
-  </si>
-  <si>
-    <t>110</t>
-  </si>
-  <si>
-    <t>CHF3</t>
-  </si>
-  <si>
-    <t>CANALINA CABLOFIL</t>
-  </si>
-  <si>
-    <t>GEMU</t>
-  </si>
-  <si>
-    <t>110X90</t>
-  </si>
-  <si>
-    <t>CL2</t>
-  </si>
-  <si>
-    <t>CARTELLA + FLANGIA (ACC+PPH)</t>
-  </si>
-  <si>
-    <t>HAMLET</t>
-  </si>
-  <si>
-    <t>1,1/2</t>
-  </si>
-  <si>
-    <t>DRDHF</t>
-  </si>
-  <si>
-    <t>CIECA</t>
-  </si>
-  <si>
-    <t>INOX</t>
-  </si>
-  <si>
-    <t>1,1/2X1</t>
-  </si>
-  <si>
-    <t>EXAC</t>
-  </si>
-  <si>
-    <t>CURVA</t>
-  </si>
-  <si>
-    <t>JACOB</t>
-  </si>
-  <si>
-    <t>1,1/2X1/2</t>
-  </si>
-  <si>
-    <t>EXHE 01</t>
-  </si>
-  <si>
-    <t>CURVE</t>
-  </si>
-  <si>
-    <t>PARKER</t>
-  </si>
-  <si>
-    <t>1,1/2X1/4</t>
-  </si>
-  <si>
-    <t>EXHE 02</t>
-  </si>
-  <si>
-    <t>DADO + FERULE ANT E POST</t>
-  </si>
-  <si>
-    <t>PFA</t>
-  </si>
-  <si>
-    <t>1,1/2X3/4</t>
-  </si>
-  <si>
-    <t>H2</t>
-  </si>
-  <si>
-    <t>FEMALE GLAND</t>
-  </si>
-  <si>
-    <t>PPH</t>
-  </si>
-  <si>
-    <t>1,1/2X38</t>
-  </si>
-  <si>
-    <t>HBr</t>
-  </si>
-  <si>
-    <t>FEMAL GLAND</t>
-  </si>
-  <si>
-    <t>PTFE</t>
-  </si>
-  <si>
-    <t>1,1/2X3/8</t>
-  </si>
-  <si>
-    <t>HeUHP</t>
-  </si>
-  <si>
-    <t>FLANGIA</t>
-  </si>
-  <si>
-    <t>PVC</t>
-  </si>
-  <si>
-    <t>1,1/2X38,1</t>
-  </si>
-  <si>
-    <t>LIM 01,,12</t>
-  </si>
-  <si>
-    <t>FLANGIA CIECA</t>
-  </si>
-  <si>
-    <t>PVDF</t>
-  </si>
-  <si>
-    <t>1,1/4</t>
+    <t>GUARNIZIONE + 8 MORSETTI</t>
+  </si>
+  <si>
+    <t>20</t>
   </si>
   <si>
     <t>N2S</t>
   </si>
   <si>
-    <t>FLANGIA CLAMP</t>
-  </si>
-  <si>
-    <t>PVDF STD</t>
-  </si>
-  <si>
-    <t>1/2</t>
+    <t>GUARNIZIONE + BULLONI</t>
+  </si>
+  <si>
+    <t>200</t>
   </si>
   <si>
     <t>N2UHP</t>
   </si>
   <si>
-    <t>FLANGIA CUSTOM</t>
-  </si>
-  <si>
-    <t>PVDF UHP</t>
-  </si>
-  <si>
-    <t>1/2X10MM (M)</t>
+    <t>HVCR MALE GLAND</t>
+  </si>
+  <si>
+    <t>200X150</t>
+  </si>
+  <si>
+    <t>N2UHP 01</t>
+  </si>
+  <si>
+    <t>MALE GLAND</t>
+  </si>
+  <si>
+    <t>20X1/2</t>
+  </si>
+  <si>
+    <t>N2UHP 02</t>
+  </si>
+  <si>
+    <t>MALE UNION</t>
+  </si>
+  <si>
+    <t>20X3/8</t>
   </si>
   <si>
     <t>NF3</t>
   </si>
   <si>
-    <t>FLANGIA DI PARTENZA DA POC</t>
-  </si>
-  <si>
-    <t>PVDF VENT</t>
-  </si>
-  <si>
-    <t>1/2X1/4</t>
+    <t>MALE UNION BSPT</t>
+  </si>
+  <si>
+    <t>25</t>
   </si>
   <si>
     <t>NG</t>
   </si>
   <si>
-    <t>FLANGIA KF</t>
-  </si>
-  <si>
-    <t>RILSAN</t>
-  </si>
-  <si>
-    <t>1/2X3/8</t>
+    <t>MANICOTTI</t>
+  </si>
+  <si>
+    <t>250</t>
   </si>
   <si>
     <t>O2STD</t>
   </si>
   <si>
-    <t>FLANGIA KF CUSTOM</t>
-  </si>
-  <si>
-    <t>SMC</t>
-  </si>
-  <si>
-    <t>1/4</t>
+    <t>MANICOTTO</t>
+  </si>
+  <si>
+    <t>250X200</t>
   </si>
   <si>
     <t>O2UHP</t>
   </si>
   <si>
-    <t>FLANGIA PP/ACC + CARTELLA + GUARN PTFE</t>
-  </si>
-  <si>
-    <t>SPECTRON</t>
-  </si>
-  <si>
-    <t>140</t>
+    <t>MANICOTTO FILETTATO</t>
+  </si>
+  <si>
+    <t>25X20</t>
+  </si>
+  <si>
+    <t>PC H2O2-01</t>
+  </si>
+  <si>
+    <t>MANOMETRO A CONTATTI</t>
+  </si>
+  <si>
+    <t>25X32</t>
+  </si>
+  <si>
+    <t>PC H2SO4</t>
+  </si>
+  <si>
+    <t>MISURATORE DI PORTATA KEYENCE FD-H</t>
+  </si>
+  <si>
+    <t>2X1</t>
+  </si>
+  <si>
+    <t>PC HCL</t>
+  </si>
+  <si>
+    <t>NIPLO FEMMINA</t>
+  </si>
+  <si>
+    <t>3</t>
+  </si>
+  <si>
+    <t>PC HF 05</t>
+  </si>
+  <si>
+    <t>NIPLO FEMMINA PVDF + TAPPO PVC</t>
+  </si>
+  <si>
+    <t>300</t>
+  </si>
+  <si>
+    <t>PC HF 49</t>
+  </si>
+  <si>
+    <t>NIPLO FEMMINA+ TAPPO PVC</t>
+  </si>
+  <si>
+    <t>300X250</t>
+  </si>
+  <si>
+    <t>PC NH4OH</t>
+  </si>
+  <si>
+    <t>ORIFIZIO CALIBRATO</t>
+  </si>
+  <si>
+    <t>315</t>
   </si>
   <si>
     <t>PCWR</t>
   </si>
   <si>
-    <t>FLANGIA TPOC</t>
-  </si>
-  <si>
-    <t>STREAS</t>
-  </si>
-  <si>
-    <t>1/4MX1/2</t>
+    <t>ORIFIZIO CALIBRATO 3 MM</t>
+  </si>
+  <si>
+    <t>32</t>
   </si>
   <si>
     <t>PCWS</t>
   </si>
   <si>
-    <t>FLK</t>
-  </si>
-  <si>
-    <t>TASSALINI</t>
-  </si>
-  <si>
-    <t>1/4X1/2</t>
+    <t>ORIFIZIO CALIBRATO 7 MM</t>
+  </si>
+  <si>
+    <t>32X1</t>
   </si>
   <si>
     <t>PV</t>
   </si>
   <si>
-    <t>FLK FEMMINA ( GHIERA GIREVOLE )</t>
-  </si>
-  <si>
-    <t>TCC</t>
-  </si>
-  <si>
-    <t>150</t>
+    <t>ORIFIZIO CALIBRATO FORATO 22 MM TASCA</t>
+  </si>
+  <si>
+    <t>32X20</t>
   </si>
   <si>
     <t>SF6</t>
   </si>
   <si>
-    <t>FLOW METER</t>
-  </si>
-  <si>
-    <t>VCR</t>
-  </si>
-  <si>
-    <t>160</t>
+    <t>ORIFIZIO CALIBRATO FORATO 25 MM TASCA</t>
+  </si>
+  <si>
+    <t>32X25</t>
   </si>
   <si>
     <t>SiCl4</t>
   </si>
   <si>
-    <t>FLOW METER CLAMPATO</t>
-  </si>
-  <si>
-    <t>ZINCATA</t>
-  </si>
-  <si>
-    <t>1"X1/2</t>
+    <t>ORIFIZIO CALIBRATO FORATO 26 MM TASCA</t>
+  </si>
+  <si>
+    <t>3/4</t>
   </si>
   <si>
     <t>SO2</t>
   </si>
   <si>
-    <t>FLUSSIMETRO CLAMPATO</t>
-  </si>
-  <si>
-    <t>1X32</t>
+    <t>ORIFIZIO CALIBRATO FORATO 32 MM TASCA</t>
+  </si>
+  <si>
+    <t>3/4X1</t>
   </si>
   <si>
     <t>SW</t>
   </si>
   <si>
-    <t>FONDELLO</t>
-  </si>
-  <si>
-    <t>1X3/4</t>
+    <t>ORIFIZIO CALIBRATO FORATO 38 MM TASCA</t>
+  </si>
+  <si>
+    <t>3/4X1/2</t>
+  </si>
+  <si>
+    <t>SW-01</t>
+  </si>
+  <si>
+    <t>ORIFIZIO CALIBRATO FORATO 48 MM TASCA</t>
+  </si>
+  <si>
+    <t>3/4X1/4</t>
+  </si>
+  <si>
+    <t>SW-02</t>
+  </si>
+  <si>
+    <t>ORIFIZIO CALIBRATO FORATO 60 MM TASCA</t>
+  </si>
+  <si>
+    <t>3/4X3/8</t>
+  </si>
+  <si>
+    <t>UPWR 01</t>
+  </si>
+  <si>
+    <t>POSIZIONAMENTO TUBO</t>
+  </si>
+  <si>
+    <t>38</t>
+  </si>
+  <si>
+    <t>UPWR-02</t>
+  </si>
+  <si>
+    <t>PROLUNGA RIDOTTA OD</t>
+  </si>
+  <si>
+    <t>3/8</t>
+  </si>
+  <si>
+    <t>UPWS-01</t>
+  </si>
+  <si>
+    <t>PUSH ON</t>
+  </si>
+  <si>
+    <t>3/8X1/4</t>
+  </si>
+  <si>
+    <t>UPWS-02</t>
+  </si>
+  <si>
+    <t>RACCORDO CUSTOM PER COLLEGAMENTO E313</t>
+  </si>
+  <si>
+    <t>40</t>
+  </si>
+  <si>
+    <t>UPWS-04</t>
+  </si>
+  <si>
+    <t>RACCORDO CUSTOM PER COLLEGAMENTO E404</t>
+  </si>
+  <si>
+    <t>40X20</t>
+  </si>
+  <si>
+    <t>UPWS-05</t>
+  </si>
+  <si>
+    <t>RACCORDO DI PASSAGGIO</t>
+  </si>
+  <si>
+    <t>40X25</t>
+  </si>
+  <si>
+    <t>UPWS-06</t>
+  </si>
+  <si>
+    <t>RACCORDO DRITTO</t>
+  </si>
+  <si>
+    <t>40X32</t>
+  </si>
+  <si>
+    <t>UPWS-07</t>
+  </si>
+  <si>
+    <t>RACCORDO FEMMINA DELLA VALVOLA CUSTOM</t>
+  </si>
+  <si>
+    <t>44,5</t>
+  </si>
+  <si>
+    <t>UPWS-08</t>
+  </si>
+  <si>
+    <t>REGOLATORE</t>
+  </si>
+  <si>
+    <t>50</t>
+  </si>
+  <si>
+    <t>UPWS-09</t>
+  </si>
+  <si>
+    <t>REGOLATORE CON MANOMETRO M/M</t>
+  </si>
+  <si>
+    <t>50X1,1/2</t>
   </si>
   <si>
     <t>VDM-01</t>
   </si>
   <si>
-    <t>GASKET INOX</t>
-  </si>
-  <si>
-    <t>1X3/8</t>
+    <t>REGOLATORE DI PRESSIONE</t>
+  </si>
+  <si>
+    <t>50X1,1/4</t>
   </si>
   <si>
     <t>VDM02</t>
   </si>
   <si>
-    <t>GASKET NICHEL</t>
-  </si>
-  <si>
-    <t>2</t>
+    <t>REGOLATORE DI PRESSIONE CLAMPATO</t>
+  </si>
+  <si>
+    <t>50X20</t>
   </si>
   <si>
     <t>VDM03</t>
   </si>
   <si>
-    <t>GUARNIZIONE + 8 MORSETTI</t>
-  </si>
-  <si>
-    <t>20</t>
+    <t>REGOLATORE DI PRESSIONE M/M</t>
+  </si>
+  <si>
+    <t>50X25</t>
   </si>
   <si>
     <t>VDM04</t>
   </si>
   <si>
-    <t>GUARNIZIONE + BULLONI</t>
-  </si>
-  <si>
-    <t>200</t>
+    <t>RIDUTTORE DI PRESSIONE</t>
+  </si>
+  <si>
+    <t>50X32</t>
   </si>
   <si>
     <t>VDM05</t>
-  </si>
-  <si>
-    <t>HVCR MALE GLAND</t>
-  </si>
-  <si>
-    <t>200X150</t>
-  </si>
-  <si>
-    <t>CT LIM</t>
-  </si>
-  <si>
-    <t>MALE GLAND</t>
-  </si>
-  <si>
-    <t>20X1/2</t>
-  </si>
-  <si>
-    <t>CT WATER</t>
-  </si>
-  <si>
-    <t>MALE UNION</t>
-  </si>
-  <si>
-    <t>20X3/8</t>
-  </si>
-  <si>
-    <t>CDA-01</t>
-  </si>
-  <si>
-    <t>MALE UNION BSPT</t>
-  </si>
-  <si>
-    <t>25</t>
-  </si>
-  <si>
-    <t>CDA-02</t>
-  </si>
-  <si>
-    <t>MANICOTTI</t>
-  </si>
-  <si>
-    <t>250</t>
-  </si>
-  <si>
-    <t>DRDA-01</t>
-  </si>
-  <si>
-    <t>MANICOTTO</t>
-  </si>
-  <si>
-    <t>250X200</t>
-  </si>
-  <si>
-    <t>DRDA-02</t>
-  </si>
-  <si>
-    <t>MANICOTTO FILETTATO</t>
-  </si>
-  <si>
-    <t>25X20</t>
-  </si>
-  <si>
-    <t>DRHF-01</t>
-  </si>
-  <si>
-    <t>MANOMETRO A CONTATTI</t>
-  </si>
-  <si>
-    <t>25X32</t>
-  </si>
-  <si>
-    <t>DRHF-02</t>
-  </si>
-  <si>
-    <t>MISURATORE DI PORTATA KEYENCE FD-H</t>
-  </si>
-  <si>
-    <t>2X1</t>
-  </si>
-  <si>
-    <t>DRNH-01</t>
-  </si>
-  <si>
-    <t>NIPLO FEMMINA</t>
-  </si>
-  <si>
-    <t>3</t>
-  </si>
-  <si>
-    <t>DRNH-02</t>
-  </si>
-  <si>
-    <t>NIPLO FEMMINA PVDF + TAPPO PVC</t>
-  </si>
-  <si>
-    <t>300</t>
-  </si>
-  <si>
-    <t>DRREC-01</t>
-  </si>
-  <si>
-    <t>NIPLO FEMMINA+ TAPPO PVC</t>
-  </si>
-  <si>
-    <t>300X250</t>
-  </si>
-  <si>
-    <t>DRSOLF</t>
-  </si>
-  <si>
-    <t>ORIFIZIO CALIBRATO</t>
-  </si>
-  <si>
-    <t>315</t>
-  </si>
-  <si>
-    <t>EXAC-01</t>
-  </si>
-  <si>
-    <t>ORIFIZIO CALIBRATO 3 MM</t>
-  </si>
-  <si>
-    <t>32</t>
-  </si>
-  <si>
-    <t>PC H2O2-01</t>
-  </si>
-  <si>
-    <t>ORIFIZIO CALIBRATO 7 MM</t>
-  </si>
-  <si>
-    <t>32X1</t>
-  </si>
-  <si>
-    <t>LIM 1…20</t>
-  </si>
-  <si>
-    <t>ORIFIZIO CALIBRATO FORATO 22 MM TASCA</t>
-  </si>
-  <si>
-    <t>32X20</t>
-  </si>
-  <si>
-    <t>N2UHP 01</t>
-  </si>
-  <si>
-    <t>ORIFIZIO CALIBRATO FORATO 25 MM TASCA</t>
-  </si>
-  <si>
-    <t>32X25</t>
-  </si>
-  <si>
-    <t>N2UHP 02</t>
-  </si>
-  <si>
-    <t>ORIFIZIO CALIBRATO FORATO 26 MM TASCA</t>
-  </si>
-  <si>
-    <t>3/4</t>
-  </si>
-  <si>
-    <t>PC H2SO4</t>
-  </si>
-  <si>
-    <t>ORIFIZIO CALIBRATO FORATO 32 MM TASCA</t>
-  </si>
-  <si>
-    <t>3/4X1</t>
-  </si>
-  <si>
-    <t>PC HCL</t>
-  </si>
-  <si>
-    <t>ORIFIZIO CALIBRATO FORATO 38 MM TASCA</t>
-  </si>
-  <si>
-    <t>3/4X1/2</t>
-  </si>
-  <si>
-    <t>PC HF 05</t>
-  </si>
-  <si>
-    <t>ORIFIZIO CALIBRATO FORATO 48 MM TASCA</t>
-  </si>
-  <si>
-    <t>3/4X1/4</t>
-  </si>
-  <si>
-    <t>PC HF 49</t>
-  </si>
-  <si>
-    <t>ORIFIZIO CALIBRATO FORATO 60 MM TASCA</t>
-  </si>
-  <si>
-    <t>3/4X3/8</t>
-  </si>
-  <si>
-    <t>PC NH4OH</t>
-  </si>
-  <si>
-    <t>POSIZIONAMENTO TUBO</t>
-  </si>
-  <si>
-    <t>38</t>
-  </si>
-  <si>
-    <t>SW-01</t>
-  </si>
-  <si>
-    <t>PROLUNGA RIDOTTA OD</t>
-  </si>
-  <si>
-    <t>3/8</t>
-  </si>
-  <si>
-    <t>SW-02</t>
-  </si>
-  <si>
-    <t>PUSH ON</t>
-  </si>
-  <si>
-    <t>3/8X1/4</t>
-  </si>
-  <si>
-    <t>UPWR 01</t>
-  </si>
-  <si>
-    <t>RACCORDO CUSTOM PER COLLEGAMENTO E313</t>
-  </si>
-  <si>
-    <t>40</t>
-  </si>
-  <si>
-    <t>UPWR-02</t>
-  </si>
-  <si>
-    <t>RACCORDO CUSTOM PER COLLEGAMENTO E404</t>
-  </si>
-  <si>
-    <t>40X20</t>
-  </si>
-  <si>
-    <t>UPWS-01</t>
-  </si>
-  <si>
-    <t>RACCORDO DI PASSAGGIO</t>
-  </si>
-  <si>
-    <t>40X25</t>
-  </si>
-  <si>
-    <t>UPWS-02</t>
-  </si>
-  <si>
-    <t>RACCORDO DRITTO</t>
-  </si>
-  <si>
-    <t>40X32</t>
-  </si>
-  <si>
-    <t>UPWS-04</t>
-  </si>
-  <si>
-    <t>RACCORDO FEMMINA DELLA VALVOLA CUSTOM</t>
-  </si>
-  <si>
-    <t>44,5</t>
-  </si>
-  <si>
-    <t>UPWS-05</t>
-  </si>
-  <si>
-    <t>REGOLATORE</t>
-  </si>
-  <si>
-    <t>50</t>
-  </si>
-  <si>
-    <t>UPWS-06</t>
-  </si>
-  <si>
-    <t>REGOLATORE CON MANOMETRO M/M</t>
-  </si>
-  <si>
-    <t>50X1,1/2</t>
-  </si>
-  <si>
-    <t>UPWS-07</t>
-  </si>
-  <si>
-    <t>REGOLATORE DI PRESSIONE</t>
-  </si>
-  <si>
-    <t>50X1,1/4</t>
-  </si>
-  <si>
-    <t>UPWS-09</t>
-  </si>
-  <si>
-    <t>REGOLATORE DI PRESSIONE CLAMPATO</t>
-  </si>
-  <si>
-    <t>50X20</t>
-  </si>
-  <si>
-    <t>UPWS-08</t>
-  </si>
-  <si>
-    <t>REGOLATORE DI PRESSIONE M/M</t>
-  </si>
-  <si>
-    <t>50X25</t>
-  </si>
-  <si>
-    <t>EXNH-01</t>
-  </si>
-  <si>
-    <t>RIDUTTORE DI PRESSIONE</t>
-  </si>
-  <si>
-    <t>50X32</t>
-  </si>
-  <si>
-    <t>EXNH02</t>
   </si>
   <si>
     <t>RIDUZIONE</t>
@@ -8343,7 +8343,6 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D501"/>
   <dataValidations count="16">
     <dataValidation type="list" allowBlank="1" sqref="A10:A501">
       <formula1>Liste!$A$2:$A$73</formula1>
@@ -9502,7 +9501,6 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D106"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>